<commit_message>
Refactor best-athlete ranks by championship
Persist official ranks on participations and refresh affected championships. Recompute report ranks on private PAthletes using the selected scoring system and mBest/wBest lists. Retire meet-wide rank storage, retain deprecated accessor aliases, and update Quebec templates and documentation.

Validate reporting and live-rank behavior with 348 passing AllTests tests. Scoreboard column changes remain a separate phase.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/competitionBook/qc/Qc_JduQ_fr_CA.xlsx
+++ b/owlcms/src/main/resources/templates/competitionBook/qc/Qc_JduQ_fr_CA.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="102">
   <si>
     <t>SITE :</t>
   </si>
@@ -204,7 +204,7 @@
     <t>${l.sinclair}</t>
   </si>
   <si>
-    <t>${l.categorySinclair}</t>
+    <t>${l.bestLifterScore}</t>
   </si>
   <si>
     <t>&lt;jx:forEach items="${wTot}" var="l" varStatus="lifterLoop"&gt;</t>
@@ -327,10 +327,10 @@
     <t>${nbAthletes}</t>
   </si>
   <si>
-    <t>&lt;jx:forEach items="${mCatSinclair}" var="l" varStatus="lifterLoop"&gt;</t>
-  </si>
-  <si>
-    <t>&lt;jx:forEach items="${wCatSinclair}" var="l" varStatus="lifterLoop"&gt;</t>
+    <t>&lt;jx:forEach items="${mBest}" var="l" varStatus="lifterLoop"&gt;</t>
+  </si>
+  <si>
+    <t>&lt;jx:forEach items="${wBest}" var="l" varStatus="lifterLoop"&gt;</t>
   </si>
   <si>
     <t>$[VLOOKUP(I12,Points!$A$2:$B$202,2)]</t>
@@ -339,10 +339,13 @@
     <t>Rank</t>
   </si>
   <si>
-    <t>${l.catSinclairRank &lt; 0 ? "inv." : (l.catSinclairRank &gt; 0 ? l.catSinclairRank : "" )}</t>
+    <t>${l.bestAthleteRank &lt; 0 ? "inv." : (l.bestAthleteRank &gt; 0 ? l.bestAthleteRank : "" )}</t>
   </si>
   <si>
     <t>${l.totalRank}</t>
+  </si>
+  <si>
+    <t>${bestRankingTitle}</t>
   </si>
 </sst>
 </file>
@@ -3650,7 +3653,7 @@
         <v>12</v>
       </c>
       <c r="S1" s="95" t="s">
-        <v>13</v>
+        <v>101</v>
       </c>
       <c r="T1" s="95"/>
       <c r="U1" s="95"/>
@@ -4796,7 +4799,7 @@
         <v>12</v>
       </c>
       <c r="S1" s="95" t="s">
-        <v>13</v>
+        <v>101</v>
       </c>
       <c r="T1" s="95"/>
       <c r="U1" s="95"/>

</xml_diff>